<commit_message>
Enhance repository with real-time multimodal deployment, online Kalman filters, and comprehensive documentation
</commit_message>
<xml_diff>
--- a/Fallall_output.xlsx
+++ b/Fallall_output.xlsx
@@ -462,20 +462,20 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>ExtraTrees</t>
+          <t>Kalman Algorithm (Improved)</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="C3" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Kalman Algorithm</t>
+          <t>Random Forest</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -512,12 +512,12 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>RandomForest_Pred</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>LSTM_Pred</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>ExtraTrees_Pred</t>
         </is>
       </c>
     </row>
@@ -526,7 +526,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C2" t="n">
         <v>1</v>
@@ -540,7 +540,7 @@
         <v>1</v>
       </c>
       <c r="B3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C3" t="n">
         <v>1</v>

</xml_diff>

<commit_message>
Integrate 5-stage presentation hierarchy, multi-sensor pipeline, FallAllD and URFD datasets
</commit_message>
<xml_diff>
--- a/Fallall_output.xlsx
+++ b/Fallall_output.xlsx
@@ -462,20 +462,20 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Kalman Algorithm (Improved)</t>
+          <t>ExtraTrees</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.3333333333333333</v>
+        <v>1</v>
       </c>
       <c r="C3" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Random Forest</t>
+          <t>Kalman Algorithm</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -512,12 +512,12 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>RandomForest_Pred</t>
+          <t>LSTM_Pred</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>LSTM_Pred</t>
+          <t>ExtraTrees_Pred</t>
         </is>
       </c>
     </row>
@@ -526,7 +526,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C2" t="n">
         <v>1</v>
@@ -540,7 +540,7 @@
         <v>1</v>
       </c>
       <c r="B3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C3" t="n">
         <v>1</v>

</xml_diff>